<commit_message>
New Change in Pulak Manch Registaration
</commit_message>
<xml_diff>
--- a/public/data/Rashtriye_Karyakarni_List.xlsx
+++ b/public/data/Rashtriye_Karyakarni_List.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\jinsharnammedia\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -879,16 +879,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.140625" style="17" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="132.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.7109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="132.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -905,7 +905,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="18">
         <v>1</v>
       </c>
@@ -922,7 +922,7 @@
         <v>9826395777</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="18">
         <v>2</v>
       </c>
@@ -939,7 +939,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="18">
         <v>3</v>
       </c>
@@ -956,7 +956,7 @@
         <v>95717004183</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="18">
         <v>4</v>
       </c>
@@ -973,7 +973,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="18">
         <v>5</v>
       </c>
@@ -990,7 +990,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="18">
         <v>6</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>9784534990</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="18">
         <v>8</v>
       </c>
@@ -1041,7 +1041,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="18">
         <v>9</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="18">
         <v>10</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>9829043342</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="18">
         <v>11</v>
       </c>
@@ -1092,7 +1092,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="18">
         <v>12</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>9810900699</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="18">
         <v>13</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="18">
         <v>14</v>
       </c>
@@ -1143,7 +1143,7 @@
         <v>9822034331</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="18">
         <v>15</v>
       </c>
@@ -1160,7 +1160,7 @@
         <v>9829116369</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="18">
         <v>16</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>9414056886</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="18">
         <v>17</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="18">
         <v>18</v>
       </c>
@@ -1211,7 +1211,7 @@
         <v>9414102255</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="18">
         <v>19</v>
       </c>
@@ -1228,7 +1228,7 @@
         <v>9829206970</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="18">
         <v>20</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>9373195054</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="18">
         <v>21</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="18">
         <v>22</v>
       </c>
@@ -1279,7 +1279,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="18">
         <v>23</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>9228555131</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="18">
         <v>24</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="18">
         <v>25</v>
       </c>
@@ -1338,16 +1338,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="132.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" style="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="132.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" style="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="13">
         <v>1</v>
       </c>
@@ -1381,7 +1381,7 @@
         <v>8120512225</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="13">
         <v>2</v>
       </c>
@@ -1398,7 +1398,7 @@
         <v>9571704183</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="13">
         <v>3</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>9869464161</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>4</v>
       </c>
@@ -1432,7 +1432,7 @@
         <v>8511188019</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="13">
         <v>5</v>
       </c>
@@ -1449,7 +1449,7 @@
         <v>9001899369</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="13">
         <v>6</v>
       </c>
@@ -1466,7 +1466,7 @@
         <v>9825800046</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="13">
         <v>7</v>
       </c>
@@ -1483,7 +1483,7 @@
         <v>9752004443</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="13">
         <v>8</v>
       </c>
@@ -1500,7 +1500,7 @@
         <v>9904450002</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="13">
         <v>9</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>9810061204</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="13">
         <v>10</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>7046321111</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
         <v>11</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="13">
         <v>12</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="13">
         <v>13</v>
       </c>
@@ -1585,7 +1585,7 @@
         <v>9425347201</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="13">
         <v>14</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="13">
         <v>15</v>
       </c>
@@ -1619,7 +1619,7 @@
         <v>7597784103</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="13">
         <v>16</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>9930959694</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="13">
         <v>17</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>8319588134</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="13">
         <v>18</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>7021162267</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="13">
         <v>19</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>9423466988</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="13">
         <v>20</v>
       </c>
@@ -1704,7 +1704,7 @@
         <v>9001202829</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="13">
         <v>21</v>
       </c>

</xml_diff>